<commit_message>
Sync planning SharePoint : S32
</commit_message>
<xml_diff>
--- a/Plannings 2026 S32.xlsx
+++ b/Plannings 2026 S32.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cdalpes.sharepoint.com/sites/msteams_bd0f90/Documents partages/02. USP - TOS - General/RH/Plannings/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{0BB1E542-A0D1-433E-BEE9-3A2D0874DD65}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="5" documentId="8_{0BB1E542-A0D1-433E-BEE9-3A2D0874DD65}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9863F60B-AC6E-47D3-9265-C8E6D2C8EAB3}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="240" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="242" uniqueCount="83">
   <si>
     <t>Planning des salariés du 03/08/2026 au 09/08/2026</t>
   </si>
@@ -265,6 +265,12 @@
   </si>
   <si>
     <t>P25F</t>
+  </si>
+  <si>
+    <t>CUP-R</t>
+  </si>
+  <si>
+    <t>13:00/18:30</t>
   </si>
 </sst>
 </file>
@@ -361,7 +367,7 @@
       <name val="Helvetica"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -376,6 +382,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFCCFFFF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF92D050"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -692,7 +704,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="46">
+  <cellXfs count="48">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -829,6 +841,12 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -945,13 +963,13 @@
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>9</xdr:row>
+      <xdr:row>10</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
       <xdr:colOff>123825</xdr:colOff>
-      <xdr:row>9</xdr:row>
+      <xdr:row>10</xdr:row>
       <xdr:rowOff>123825</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -989,13 +1007,13 @@
     <xdr:from>
       <xdr:col>2</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>9</xdr:row>
+      <xdr:row>10</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
       <xdr:colOff>123825</xdr:colOff>
-      <xdr:row>9</xdr:row>
+      <xdr:row>10</xdr:row>
       <xdr:rowOff>123825</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -1033,13 +1051,13 @@
     <xdr:from>
       <xdr:col>3</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>9</xdr:row>
+      <xdr:row>10</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
       <xdr:colOff>123825</xdr:colOff>
-      <xdr:row>9</xdr:row>
+      <xdr:row>10</xdr:row>
       <xdr:rowOff>123825</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -1077,13 +1095,13 @@
     <xdr:from>
       <xdr:col>4</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>9</xdr:row>
+      <xdr:row>10</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>4</xdr:col>
       <xdr:colOff>123825</xdr:colOff>
-      <xdr:row>9</xdr:row>
+      <xdr:row>10</xdr:row>
       <xdr:rowOff>123825</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -1121,13 +1139,13 @@
     <xdr:from>
       <xdr:col>5</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>9</xdr:row>
+      <xdr:row>10</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>5</xdr:col>
       <xdr:colOff>123825</xdr:colOff>
-      <xdr:row>9</xdr:row>
+      <xdr:row>10</xdr:row>
       <xdr:rowOff>123825</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -1165,13 +1183,13 @@
     <xdr:from>
       <xdr:col>3</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>15</xdr:row>
+      <xdr:row>16</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
       <xdr:colOff>123825</xdr:colOff>
-      <xdr:row>15</xdr:row>
+      <xdr:row>16</xdr:row>
       <xdr:rowOff>123825</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -1209,13 +1227,13 @@
     <xdr:from>
       <xdr:col>5</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>15</xdr:row>
+      <xdr:row>16</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>5</xdr:col>
       <xdr:colOff>123825</xdr:colOff>
-      <xdr:row>15</xdr:row>
+      <xdr:row>16</xdr:row>
       <xdr:rowOff>123825</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -1253,13 +1271,13 @@
     <xdr:from>
       <xdr:col>7</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>15</xdr:row>
+      <xdr:row>16</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>123825</xdr:colOff>
-      <xdr:row>15</xdr:row>
+      <xdr:row>16</xdr:row>
       <xdr:rowOff>123825</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -1297,13 +1315,13 @@
     <xdr:from>
       <xdr:col>4</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>19</xdr:row>
+      <xdr:row>20</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>4</xdr:col>
       <xdr:colOff>123825</xdr:colOff>
-      <xdr:row>19</xdr:row>
+      <xdr:row>20</xdr:row>
       <xdr:rowOff>123825</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -1341,13 +1359,13 @@
     <xdr:from>
       <xdr:col>5</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>19</xdr:row>
+      <xdr:row>20</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>5</xdr:col>
       <xdr:colOff>123825</xdr:colOff>
-      <xdr:row>19</xdr:row>
+      <xdr:row>20</xdr:row>
       <xdr:rowOff>123825</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -1385,13 +1403,13 @@
     <xdr:from>
       <xdr:col>6</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>19</xdr:row>
+      <xdr:row>20</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>6</xdr:col>
       <xdr:colOff>123825</xdr:colOff>
-      <xdr:row>19</xdr:row>
+      <xdr:row>20</xdr:row>
       <xdr:rowOff>123825</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -1429,13 +1447,13 @@
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>22</xdr:row>
+      <xdr:row>23</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
       <xdr:colOff>123825</xdr:colOff>
-      <xdr:row>22</xdr:row>
+      <xdr:row>23</xdr:row>
       <xdr:rowOff>123825</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -1473,13 +1491,13 @@
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>24</xdr:row>
+      <xdr:row>25</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
       <xdr:colOff>123825</xdr:colOff>
-      <xdr:row>24</xdr:row>
+      <xdr:row>25</xdr:row>
       <xdr:rowOff>123825</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -1517,13 +1535,13 @@
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>26</xdr:row>
+      <xdr:row>27</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
       <xdr:colOff>123825</xdr:colOff>
-      <xdr:row>26</xdr:row>
+      <xdr:row>27</xdr:row>
       <xdr:rowOff>123825</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -1561,13 +1579,13 @@
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>28</xdr:row>
+      <xdr:row>29</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
       <xdr:colOff>123825</xdr:colOff>
-      <xdr:row>28</xdr:row>
+      <xdr:row>29</xdr:row>
       <xdr:rowOff>123825</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -1605,13 +1623,13 @@
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>30</xdr:row>
+      <xdr:row>31</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
       <xdr:colOff>123825</xdr:colOff>
-      <xdr:row>30</xdr:row>
+      <xdr:row>31</xdr:row>
       <xdr:rowOff>123825</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -1649,13 +1667,13 @@
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>32</xdr:row>
+      <xdr:row>33</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
       <xdr:colOff>123825</xdr:colOff>
-      <xdr:row>32</xdr:row>
+      <xdr:row>33</xdr:row>
       <xdr:rowOff>123825</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -1693,13 +1711,13 @@
     <xdr:from>
       <xdr:col>2</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>22</xdr:row>
+      <xdr:row>23</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
       <xdr:colOff>123825</xdr:colOff>
-      <xdr:row>22</xdr:row>
+      <xdr:row>23</xdr:row>
       <xdr:rowOff>123825</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -1737,13 +1755,13 @@
     <xdr:from>
       <xdr:col>2</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>24</xdr:row>
+      <xdr:row>25</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
       <xdr:colOff>123825</xdr:colOff>
-      <xdr:row>24</xdr:row>
+      <xdr:row>25</xdr:row>
       <xdr:rowOff>123825</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -1781,13 +1799,13 @@
     <xdr:from>
       <xdr:col>2</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>26</xdr:row>
+      <xdr:row>27</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
       <xdr:colOff>123825</xdr:colOff>
-      <xdr:row>26</xdr:row>
+      <xdr:row>27</xdr:row>
       <xdr:rowOff>123825</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -1825,13 +1843,13 @@
     <xdr:from>
       <xdr:col>2</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>28</xdr:row>
+      <xdr:row>29</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
       <xdr:colOff>123825</xdr:colOff>
-      <xdr:row>28</xdr:row>
+      <xdr:row>29</xdr:row>
       <xdr:rowOff>123825</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -1869,13 +1887,13 @@
     <xdr:from>
       <xdr:col>2</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>30</xdr:row>
+      <xdr:row>31</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
       <xdr:colOff>123825</xdr:colOff>
-      <xdr:row>30</xdr:row>
+      <xdr:row>31</xdr:row>
       <xdr:rowOff>123825</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -1913,13 +1931,13 @@
     <xdr:from>
       <xdr:col>3</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>22</xdr:row>
+      <xdr:row>23</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
       <xdr:colOff>123825</xdr:colOff>
-      <xdr:row>22</xdr:row>
+      <xdr:row>23</xdr:row>
       <xdr:rowOff>123825</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -1957,13 +1975,13 @@
     <xdr:from>
       <xdr:col>3</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>24</xdr:row>
+      <xdr:row>25</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
       <xdr:colOff>123825</xdr:colOff>
-      <xdr:row>24</xdr:row>
+      <xdr:row>25</xdr:row>
       <xdr:rowOff>123825</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -2001,13 +2019,13 @@
     <xdr:from>
       <xdr:col>3</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>26</xdr:row>
+      <xdr:row>27</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
       <xdr:colOff>123825</xdr:colOff>
-      <xdr:row>26</xdr:row>
+      <xdr:row>27</xdr:row>
       <xdr:rowOff>123825</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -2045,13 +2063,13 @@
     <xdr:from>
       <xdr:col>3</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>28</xdr:row>
+      <xdr:row>29</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
       <xdr:colOff>123825</xdr:colOff>
-      <xdr:row>28</xdr:row>
+      <xdr:row>29</xdr:row>
       <xdr:rowOff>123825</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -2089,13 +2107,13 @@
     <xdr:from>
       <xdr:col>3</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>30</xdr:row>
+      <xdr:row>31</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
       <xdr:colOff>123825</xdr:colOff>
-      <xdr:row>30</xdr:row>
+      <xdr:row>31</xdr:row>
       <xdr:rowOff>123825</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -2133,13 +2151,13 @@
     <xdr:from>
       <xdr:col>3</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>32</xdr:row>
+      <xdr:row>33</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
       <xdr:colOff>123825</xdr:colOff>
-      <xdr:row>32</xdr:row>
+      <xdr:row>33</xdr:row>
       <xdr:rowOff>123825</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -2177,13 +2195,13 @@
     <xdr:from>
       <xdr:col>4</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>22</xdr:row>
+      <xdr:row>23</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>4</xdr:col>
       <xdr:colOff>123825</xdr:colOff>
-      <xdr:row>22</xdr:row>
+      <xdr:row>23</xdr:row>
       <xdr:rowOff>123825</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -2221,13 +2239,13 @@
     <xdr:from>
       <xdr:col>4</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>24</xdr:row>
+      <xdr:row>25</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>4</xdr:col>
       <xdr:colOff>123825</xdr:colOff>
-      <xdr:row>24</xdr:row>
+      <xdr:row>25</xdr:row>
       <xdr:rowOff>123825</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -2265,13 +2283,13 @@
     <xdr:from>
       <xdr:col>4</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>26</xdr:row>
+      <xdr:row>27</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>4</xdr:col>
       <xdr:colOff>123825</xdr:colOff>
-      <xdr:row>26</xdr:row>
+      <xdr:row>27</xdr:row>
       <xdr:rowOff>123825</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -2309,13 +2327,13 @@
     <xdr:from>
       <xdr:col>4</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>28</xdr:row>
+      <xdr:row>29</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>4</xdr:col>
       <xdr:colOff>123825</xdr:colOff>
-      <xdr:row>28</xdr:row>
+      <xdr:row>29</xdr:row>
       <xdr:rowOff>123825</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -2353,13 +2371,13 @@
     <xdr:from>
       <xdr:col>4</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>30</xdr:row>
+      <xdr:row>31</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>4</xdr:col>
       <xdr:colOff>123825</xdr:colOff>
-      <xdr:row>30</xdr:row>
+      <xdr:row>31</xdr:row>
       <xdr:rowOff>123825</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -2397,13 +2415,13 @@
     <xdr:from>
       <xdr:col>5</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>22</xdr:row>
+      <xdr:row>23</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>5</xdr:col>
       <xdr:colOff>123825</xdr:colOff>
-      <xdr:row>22</xdr:row>
+      <xdr:row>23</xdr:row>
       <xdr:rowOff>123825</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -2441,13 +2459,13 @@
     <xdr:from>
       <xdr:col>5</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>24</xdr:row>
+      <xdr:row>25</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>5</xdr:col>
       <xdr:colOff>123825</xdr:colOff>
-      <xdr:row>24</xdr:row>
+      <xdr:row>25</xdr:row>
       <xdr:rowOff>123825</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -2485,13 +2503,13 @@
     <xdr:from>
       <xdr:col>5</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>26</xdr:row>
+      <xdr:row>27</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>5</xdr:col>
       <xdr:colOff>123825</xdr:colOff>
-      <xdr:row>26</xdr:row>
+      <xdr:row>27</xdr:row>
       <xdr:rowOff>123825</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -2529,13 +2547,13 @@
     <xdr:from>
       <xdr:col>5</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>28</xdr:row>
+      <xdr:row>29</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>5</xdr:col>
       <xdr:colOff>123825</xdr:colOff>
-      <xdr:row>28</xdr:row>
+      <xdr:row>29</xdr:row>
       <xdr:rowOff>123825</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -2573,13 +2591,13 @@
     <xdr:from>
       <xdr:col>5</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>30</xdr:row>
+      <xdr:row>31</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>5</xdr:col>
       <xdr:colOff>123825</xdr:colOff>
-      <xdr:row>30</xdr:row>
+      <xdr:row>31</xdr:row>
       <xdr:rowOff>123825</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -2617,13 +2635,13 @@
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>34</xdr:row>
+      <xdr:row>35</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
       <xdr:colOff>123825</xdr:colOff>
-      <xdr:row>34</xdr:row>
+      <xdr:row>35</xdr:row>
       <xdr:rowOff>123825</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -2661,13 +2679,13 @@
     <xdr:from>
       <xdr:col>4</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>34</xdr:row>
+      <xdr:row>35</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>4</xdr:col>
       <xdr:colOff>123825</xdr:colOff>
-      <xdr:row>34</xdr:row>
+      <xdr:row>35</xdr:row>
       <xdr:rowOff>123825</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -2705,13 +2723,13 @@
     <xdr:from>
       <xdr:col>2</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>36</xdr:row>
+      <xdr:row>37</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
       <xdr:colOff>123825</xdr:colOff>
-      <xdr:row>36</xdr:row>
+      <xdr:row>37</xdr:row>
       <xdr:rowOff>123825</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -2749,13 +2767,13 @@
     <xdr:from>
       <xdr:col>6</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>36</xdr:row>
+      <xdr:row>37</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>6</xdr:col>
       <xdr:colOff>123825</xdr:colOff>
-      <xdr:row>36</xdr:row>
+      <xdr:row>37</xdr:row>
       <xdr:rowOff>123825</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -2793,13 +2811,13 @@
     <xdr:from>
       <xdr:col>7</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>36</xdr:row>
+      <xdr:row>37</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>123825</xdr:colOff>
-      <xdr:row>36</xdr:row>
+      <xdr:row>37</xdr:row>
       <xdr:rowOff>123825</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -2837,13 +2855,13 @@
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>41</xdr:row>
+      <xdr:row>42</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
       <xdr:colOff>123825</xdr:colOff>
-      <xdr:row>41</xdr:row>
+      <xdr:row>42</xdr:row>
       <xdr:rowOff>123825</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -2881,13 +2899,13 @@
     <xdr:from>
       <xdr:col>2</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>41</xdr:row>
+      <xdr:row>42</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
       <xdr:colOff>123825</xdr:colOff>
-      <xdr:row>41</xdr:row>
+      <xdr:row>42</xdr:row>
       <xdr:rowOff>123825</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -2925,13 +2943,13 @@
     <xdr:from>
       <xdr:col>3</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>41</xdr:row>
+      <xdr:row>42</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
       <xdr:colOff>123825</xdr:colOff>
-      <xdr:row>41</xdr:row>
+      <xdr:row>42</xdr:row>
       <xdr:rowOff>123825</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -2969,13 +2987,13 @@
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>44</xdr:row>
+      <xdr:row>45</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
       <xdr:colOff>123825</xdr:colOff>
-      <xdr:row>44</xdr:row>
+      <xdr:row>45</xdr:row>
       <xdr:rowOff>123825</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -3013,13 +3031,13 @@
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>46</xdr:row>
+      <xdr:row>47</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
       <xdr:colOff>123825</xdr:colOff>
-      <xdr:row>46</xdr:row>
+      <xdr:row>47</xdr:row>
       <xdr:rowOff>123825</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -3057,13 +3075,13 @@
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>48</xdr:row>
+      <xdr:row>49</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
       <xdr:colOff>123825</xdr:colOff>
-      <xdr:row>48</xdr:row>
+      <xdr:row>49</xdr:row>
       <xdr:rowOff>123825</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -3101,13 +3119,13 @@
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>50</xdr:row>
+      <xdr:row>51</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
       <xdr:colOff>123825</xdr:colOff>
-      <xdr:row>50</xdr:row>
+      <xdr:row>51</xdr:row>
       <xdr:rowOff>123825</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -3145,13 +3163,13 @@
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>52</xdr:row>
+      <xdr:row>53</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
       <xdr:colOff>123825</xdr:colOff>
-      <xdr:row>52</xdr:row>
+      <xdr:row>53</xdr:row>
       <xdr:rowOff>123825</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -3189,13 +3207,13 @@
     <xdr:from>
       <xdr:col>2</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>44</xdr:row>
+      <xdr:row>45</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
       <xdr:colOff>123825</xdr:colOff>
-      <xdr:row>44</xdr:row>
+      <xdr:row>45</xdr:row>
       <xdr:rowOff>123825</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -3233,13 +3251,13 @@
     <xdr:from>
       <xdr:col>2</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>46</xdr:row>
+      <xdr:row>47</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
       <xdr:colOff>123825</xdr:colOff>
-      <xdr:row>46</xdr:row>
+      <xdr:row>47</xdr:row>
       <xdr:rowOff>123825</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -3277,13 +3295,13 @@
     <xdr:from>
       <xdr:col>2</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>48</xdr:row>
+      <xdr:row>49</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
       <xdr:colOff>123825</xdr:colOff>
-      <xdr:row>48</xdr:row>
+      <xdr:row>49</xdr:row>
       <xdr:rowOff>123825</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -3321,13 +3339,13 @@
     <xdr:from>
       <xdr:col>2</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>50</xdr:row>
+      <xdr:row>51</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
       <xdr:colOff>123825</xdr:colOff>
-      <xdr:row>50</xdr:row>
+      <xdr:row>51</xdr:row>
       <xdr:rowOff>123825</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -3365,13 +3383,13 @@
     <xdr:from>
       <xdr:col>2</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>52</xdr:row>
+      <xdr:row>53</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
       <xdr:colOff>123825</xdr:colOff>
-      <xdr:row>52</xdr:row>
+      <xdr:row>53</xdr:row>
       <xdr:rowOff>123825</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -3409,13 +3427,13 @@
     <xdr:from>
       <xdr:col>2</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>54</xdr:row>
+      <xdr:row>55</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
       <xdr:colOff>123825</xdr:colOff>
-      <xdr:row>54</xdr:row>
+      <xdr:row>55</xdr:row>
       <xdr:rowOff>123825</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -3453,13 +3471,13 @@
     <xdr:from>
       <xdr:col>3</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>44</xdr:row>
+      <xdr:row>45</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
       <xdr:colOff>123825</xdr:colOff>
-      <xdr:row>44</xdr:row>
+      <xdr:row>45</xdr:row>
       <xdr:rowOff>123825</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -3497,13 +3515,13 @@
     <xdr:from>
       <xdr:col>3</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>46</xdr:row>
+      <xdr:row>47</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
       <xdr:colOff>123825</xdr:colOff>
-      <xdr:row>46</xdr:row>
+      <xdr:row>47</xdr:row>
       <xdr:rowOff>123825</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -3541,13 +3559,13 @@
     <xdr:from>
       <xdr:col>3</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>48</xdr:row>
+      <xdr:row>49</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
       <xdr:colOff>123825</xdr:colOff>
-      <xdr:row>48</xdr:row>
+      <xdr:row>49</xdr:row>
       <xdr:rowOff>123825</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -3585,13 +3603,13 @@
     <xdr:from>
       <xdr:col>3</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>50</xdr:row>
+      <xdr:row>51</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
       <xdr:colOff>123825</xdr:colOff>
-      <xdr:row>50</xdr:row>
+      <xdr:row>51</xdr:row>
       <xdr:rowOff>123825</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -3629,13 +3647,13 @@
     <xdr:from>
       <xdr:col>3</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>52</xdr:row>
+      <xdr:row>53</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
       <xdr:colOff>123825</xdr:colOff>
-      <xdr:row>52</xdr:row>
+      <xdr:row>53</xdr:row>
       <xdr:rowOff>123825</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -3673,13 +3691,13 @@
     <xdr:from>
       <xdr:col>4</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>44</xdr:row>
+      <xdr:row>45</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>4</xdr:col>
       <xdr:colOff>123825</xdr:colOff>
-      <xdr:row>44</xdr:row>
+      <xdr:row>45</xdr:row>
       <xdr:rowOff>123825</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -3717,13 +3735,13 @@
     <xdr:from>
       <xdr:col>4</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>46</xdr:row>
+      <xdr:row>47</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>4</xdr:col>
       <xdr:colOff>123825</xdr:colOff>
-      <xdr:row>46</xdr:row>
+      <xdr:row>47</xdr:row>
       <xdr:rowOff>123825</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -3761,13 +3779,13 @@
     <xdr:from>
       <xdr:col>4</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>48</xdr:row>
+      <xdr:row>49</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>4</xdr:col>
       <xdr:colOff>123825</xdr:colOff>
-      <xdr:row>48</xdr:row>
+      <xdr:row>49</xdr:row>
       <xdr:rowOff>123825</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -3805,13 +3823,13 @@
     <xdr:from>
       <xdr:col>4</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>50</xdr:row>
+      <xdr:row>51</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>4</xdr:col>
       <xdr:colOff>123825</xdr:colOff>
-      <xdr:row>50</xdr:row>
+      <xdr:row>51</xdr:row>
       <xdr:rowOff>123825</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -3849,13 +3867,13 @@
     <xdr:from>
       <xdr:col>4</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>52</xdr:row>
+      <xdr:row>53</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>4</xdr:col>
       <xdr:colOff>123825</xdr:colOff>
-      <xdr:row>52</xdr:row>
+      <xdr:row>53</xdr:row>
       <xdr:rowOff>123825</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -3893,13 +3911,13 @@
     <xdr:from>
       <xdr:col>4</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>54</xdr:row>
+      <xdr:row>55</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>4</xdr:col>
       <xdr:colOff>123825</xdr:colOff>
-      <xdr:row>54</xdr:row>
+      <xdr:row>55</xdr:row>
       <xdr:rowOff>123825</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -3937,13 +3955,13 @@
     <xdr:from>
       <xdr:col>5</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>44</xdr:row>
+      <xdr:row>45</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>5</xdr:col>
       <xdr:colOff>123825</xdr:colOff>
-      <xdr:row>44</xdr:row>
+      <xdr:row>45</xdr:row>
       <xdr:rowOff>123825</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -3981,13 +3999,13 @@
     <xdr:from>
       <xdr:col>5</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>46</xdr:row>
+      <xdr:row>47</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>5</xdr:col>
       <xdr:colOff>123825</xdr:colOff>
-      <xdr:row>46</xdr:row>
+      <xdr:row>47</xdr:row>
       <xdr:rowOff>123825</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -4025,13 +4043,13 @@
     <xdr:from>
       <xdr:col>5</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>48</xdr:row>
+      <xdr:row>49</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>5</xdr:col>
       <xdr:colOff>123825</xdr:colOff>
-      <xdr:row>48</xdr:row>
+      <xdr:row>49</xdr:row>
       <xdr:rowOff>123825</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -4069,13 +4087,13 @@
     <xdr:from>
       <xdr:col>5</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>50</xdr:row>
+      <xdr:row>51</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>5</xdr:col>
       <xdr:colOff>123825</xdr:colOff>
-      <xdr:row>50</xdr:row>
+      <xdr:row>51</xdr:row>
       <xdr:rowOff>123825</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -4113,13 +4131,13 @@
     <xdr:from>
       <xdr:col>5</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>52</xdr:row>
+      <xdr:row>53</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>5</xdr:col>
       <xdr:colOff>123825</xdr:colOff>
-      <xdr:row>52</xdr:row>
+      <xdr:row>53</xdr:row>
       <xdr:rowOff>123825</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -4144,6 +4162,50 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
+          <a:ext cx="123825" cy="123825"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>123825</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>123825</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="77" name="Picture 1" descr="Picture">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{07ECA38A-09EE-4FEC-B05B-8A4DD96A94FA}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3657600" y="3438525"/>
           <a:ext cx="123825" cy="123825"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -4525,7 +4587,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H59"/>
+  <dimension ref="A1:H60"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="8" width="31.28515625" customWidth="1"/>
@@ -4656,79 +4718,79 @@
       <c r="G8" s="17"/>
       <c r="H8" s="18"/>
     </row>
-    <row r="9" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="15" t="s">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A9" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="B9" s="16"/>
-      <c r="C9" s="17"/>
-      <c r="D9" s="17"/>
-      <c r="E9" s="17"/>
-      <c r="F9" s="17"/>
-      <c r="G9" s="17"/>
-      <c r="H9" s="18"/>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A10" s="19" t="s">
+      <c r="B9" s="20"/>
+      <c r="C9" s="20"/>
+      <c r="D9" s="20"/>
+      <c r="E9" s="20"/>
+      <c r="F9" s="20"/>
+      <c r="G9" s="46" t="s">
+        <v>81</v>
+      </c>
+      <c r="H9" s="21"/>
+    </row>
+    <row r="10" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="24"/>
+      <c r="B10" s="25"/>
+      <c r="C10" s="25"/>
+      <c r="D10" s="25"/>
+      <c r="E10" s="25"/>
+      <c r="F10" s="25"/>
+      <c r="G10" s="47" t="s">
+        <v>82</v>
+      </c>
+      <c r="H10" s="26"/>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A11" s="19" t="s">
         <v>18</v>
       </c>
-      <c r="B10" s="20" t="s">
+      <c r="B11" s="20" t="s">
         <v>12</v>
       </c>
-      <c r="C10" s="20" t="s">
+      <c r="C11" s="20" t="s">
         <v>12</v>
       </c>
-      <c r="D10" s="20" t="s">
+      <c r="D11" s="20" t="s">
         <v>12</v>
       </c>
-      <c r="E10" s="20" t="s">
+      <c r="E11" s="20" t="s">
         <v>12</v>
       </c>
-      <c r="F10" s="20" t="s">
+      <c r="F11" s="20" t="s">
         <v>12</v>
       </c>
-      <c r="G10" s="20"/>
-      <c r="H10" s="21"/>
-    </row>
-    <row r="11" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="24"/>
-      <c r="B11" s="25" t="s">
+      <c r="G11" s="20"/>
+      <c r="H11" s="21"/>
+    </row>
+    <row r="12" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="24"/>
+      <c r="B12" s="25" t="s">
         <v>19</v>
       </c>
-      <c r="C11" s="25" t="s">
+      <c r="C12" s="25" t="s">
         <v>20</v>
       </c>
-      <c r="D11" s="25" t="s">
+      <c r="D12" s="25" t="s">
         <v>21</v>
       </c>
-      <c r="E11" s="25" t="s">
+      <c r="E12" s="25" t="s">
         <v>22</v>
       </c>
-      <c r="F11" s="25" t="s">
+      <c r="F12" s="25" t="s">
         <v>22</v>
       </c>
-      <c r="G11" s="25"/>
-      <c r="H11" s="26"/>
-    </row>
-    <row r="12" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="15" t="s">
-        <v>23</v>
-      </c>
-      <c r="B12" s="16"/>
-      <c r="C12" s="17"/>
-      <c r="D12" s="17"/>
-      <c r="E12" s="17"/>
-      <c r="F12" s="17"/>
-      <c r="G12" s="17"/>
-      <c r="H12" s="18"/>
+      <c r="G12" s="25"/>
+      <c r="H12" s="26"/>
     </row>
     <row r="13" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="15" t="s">
-        <v>24</v>
-      </c>
-      <c r="B13" s="16" t="s">
-        <v>78</v>
-      </c>
+        <v>23</v>
+      </c>
+      <c r="B13" s="16"/>
       <c r="C13" s="17"/>
       <c r="D13" s="17"/>
       <c r="E13" s="17"/>
@@ -4738,9 +4800,11 @@
     </row>
     <row r="14" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="15" t="s">
-        <v>25</v>
-      </c>
-      <c r="B14" s="16"/>
+        <v>24</v>
+      </c>
+      <c r="B14" s="16" t="s">
+        <v>78</v>
+      </c>
       <c r="C14" s="17"/>
       <c r="D14" s="17"/>
       <c r="E14" s="17"/>
@@ -4750,11 +4814,9 @@
     </row>
     <row r="15" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="15" t="s">
-        <v>26</v>
-      </c>
-      <c r="B15" s="16" t="s">
-        <v>78</v>
-      </c>
+        <v>25</v>
+      </c>
+      <c r="B15" s="16"/>
       <c r="C15" s="17"/>
       <c r="D15" s="17"/>
       <c r="E15" s="17"/>
@@ -4762,55 +4824,57 @@
       <c r="G15" s="17"/>
       <c r="H15" s="18"/>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A16" s="19" t="s">
+    <row r="16" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="15" t="s">
+        <v>26</v>
+      </c>
+      <c r="B16" s="16" t="s">
+        <v>78</v>
+      </c>
+      <c r="C16" s="17"/>
+      <c r="D16" s="17"/>
+      <c r="E16" s="17"/>
+      <c r="F16" s="17"/>
+      <c r="G16" s="17"/>
+      <c r="H16" s="18"/>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A17" s="19" t="s">
         <v>27</v>
       </c>
-      <c r="B16" s="20"/>
-      <c r="C16" s="20"/>
-      <c r="D16" s="20" t="s">
+      <c r="B17" s="20"/>
+      <c r="C17" s="20"/>
+      <c r="D17" s="20" t="s">
         <v>12</v>
       </c>
-      <c r="E16" s="20"/>
-      <c r="F16" s="20" t="s">
+      <c r="E17" s="20"/>
+      <c r="F17" s="20" t="s">
         <v>12</v>
       </c>
-      <c r="G16" s="20"/>
-      <c r="H16" s="21" t="s">
+      <c r="G17" s="20"/>
+      <c r="H17" s="21" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="17" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="33"/>
-      <c r="B17" s="1"/>
-      <c r="C17" s="1"/>
-      <c r="D17" s="1" t="s">
+    <row r="18" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="33"/>
+      <c r="B18" s="1"/>
+      <c r="C18" s="1"/>
+      <c r="D18" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="E17" s="1"/>
-      <c r="F17" s="1" t="s">
+      <c r="E18" s="1"/>
+      <c r="F18" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="G17" s="1"/>
-      <c r="H17" s="23" t="s">
+      <c r="G18" s="1"/>
+      <c r="H18" s="23" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="18" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="15" t="s">
-        <v>32</v>
-      </c>
-      <c r="B18" s="27"/>
-      <c r="C18" s="28"/>
-      <c r="D18" s="28"/>
-      <c r="E18" s="28"/>
-      <c r="F18" s="28"/>
-      <c r="G18" s="28"/>
-      <c r="H18" s="29"/>
     </row>
     <row r="19" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="15" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B19" s="27"/>
       <c r="C19" s="28"/>
@@ -4820,373 +4884,373 @@
       <c r="G19" s="28"/>
       <c r="H19" s="29"/>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A20" s="19" t="s">
+    <row r="20" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="15" t="s">
+        <v>33</v>
+      </c>
+      <c r="B20" s="27"/>
+      <c r="C20" s="28"/>
+      <c r="D20" s="28"/>
+      <c r="E20" s="28"/>
+      <c r="F20" s="28"/>
+      <c r="G20" s="28"/>
+      <c r="H20" s="29"/>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A21" s="19" t="s">
         <v>34</v>
       </c>
-      <c r="B20" s="20"/>
-      <c r="C20" s="20"/>
-      <c r="D20" s="20"/>
-      <c r="E20" s="20" t="s">
+      <c r="B21" s="20"/>
+      <c r="C21" s="20"/>
+      <c r="D21" s="20"/>
+      <c r="E21" s="20" t="s">
         <v>12</v>
       </c>
-      <c r="F20" s="20" t="s">
+      <c r="F21" s="20" t="s">
         <v>12</v>
       </c>
-      <c r="G20" s="20" t="s">
+      <c r="G21" s="20" t="s">
         <v>12</v>
       </c>
-      <c r="H20" s="21"/>
-    </row>
-    <row r="21" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="24"/>
-      <c r="B21" s="25"/>
-      <c r="C21" s="25"/>
-      <c r="D21" s="25"/>
-      <c r="E21" s="25" t="s">
+      <c r="H21" s="21"/>
+    </row>
+    <row r="22" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A22" s="24"/>
+      <c r="B22" s="25"/>
+      <c r="C22" s="25"/>
+      <c r="D22" s="25"/>
+      <c r="E22" s="25" t="s">
         <v>35</v>
       </c>
-      <c r="F21" s="25" t="s">
+      <c r="F22" s="25" t="s">
         <v>35</v>
       </c>
-      <c r="G21" s="25" t="s">
+      <c r="G22" s="25" t="s">
         <v>30</v>
       </c>
-      <c r="H21" s="26"/>
-    </row>
-    <row r="22" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="34" t="s">
+      <c r="H22" s="26"/>
+    </row>
+    <row r="23" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A23" s="34" t="s">
         <v>36</v>
       </c>
-      <c r="B22" s="35"/>
-      <c r="C22" s="36"/>
-      <c r="D22" s="36"/>
-      <c r="E22" s="36"/>
-      <c r="F22" s="36"/>
-      <c r="G22" s="36"/>
-      <c r="H22" s="37"/>
-    </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A23" s="19" t="s">
+      <c r="B23" s="35"/>
+      <c r="C23" s="36"/>
+      <c r="D23" s="36"/>
+      <c r="E23" s="36"/>
+      <c r="F23" s="36"/>
+      <c r="G23" s="36"/>
+      <c r="H23" s="37"/>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A24" s="19" t="s">
         <v>37</v>
       </c>
-      <c r="B23" s="42" t="s">
+      <c r="B24" s="42" t="s">
         <v>38</v>
       </c>
-      <c r="C23" s="42" t="s">
+      <c r="C24" s="42" t="s">
         <v>38</v>
       </c>
-      <c r="D23" s="42" t="s">
+      <c r="D24" s="42" t="s">
         <v>38</v>
       </c>
-      <c r="E23" s="42" t="s">
+      <c r="E24" s="42" t="s">
         <v>38</v>
       </c>
-      <c r="F23" s="42" t="s">
+      <c r="F24" s="42" t="s">
         <v>38</v>
       </c>
-      <c r="G23" s="20"/>
-      <c r="H23" s="21"/>
-    </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A24" s="22"/>
-      <c r="B24" s="43" t="s">
-        <v>39</v>
-      </c>
-      <c r="C24" s="43" t="s">
-        <v>39</v>
-      </c>
-      <c r="D24" s="43" t="s">
-        <v>40</v>
-      </c>
-      <c r="E24" s="43" t="s">
-        <v>39</v>
-      </c>
-      <c r="F24" s="43" t="s">
-        <v>40</v>
-      </c>
-      <c r="G24" s="1"/>
-      <c r="H24" s="23"/>
+      <c r="G24" s="20"/>
+      <c r="H24" s="21"/>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A25" s="22"/>
-      <c r="B25" s="44" t="s">
-        <v>41</v>
-      </c>
-      <c r="C25" s="44" t="s">
-        <v>41</v>
-      </c>
-      <c r="D25" s="44" t="s">
-        <v>41</v>
-      </c>
-      <c r="E25" s="44" t="s">
-        <v>41</v>
-      </c>
-      <c r="F25" s="44" t="s">
-        <v>41</v>
+      <c r="B25" s="43" t="s">
+        <v>39</v>
+      </c>
+      <c r="C25" s="43" t="s">
+        <v>39</v>
+      </c>
+      <c r="D25" s="43" t="s">
+        <v>40</v>
+      </c>
+      <c r="E25" s="43" t="s">
+        <v>39</v>
+      </c>
+      <c r="F25" s="43" t="s">
+        <v>40</v>
       </c>
       <c r="G25" s="1"/>
       <c r="H25" s="23"/>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A26" s="22"/>
-      <c r="B26" s="43" t="s">
-        <v>42</v>
-      </c>
-      <c r="C26" s="43" t="s">
-        <v>42</v>
-      </c>
-      <c r="D26" s="43" t="s">
-        <v>42</v>
-      </c>
-      <c r="E26" s="43" t="s">
-        <v>42</v>
-      </c>
-      <c r="F26" s="43" t="s">
-        <v>42</v>
+      <c r="B26" s="44" t="s">
+        <v>41</v>
+      </c>
+      <c r="C26" s="44" t="s">
+        <v>41</v>
+      </c>
+      <c r="D26" s="44" t="s">
+        <v>41</v>
+      </c>
+      <c r="E26" s="44" t="s">
+        <v>41</v>
+      </c>
+      <c r="F26" s="44" t="s">
+        <v>41</v>
       </c>
       <c r="G26" s="1"/>
       <c r="H26" s="23"/>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A27" s="22"/>
-      <c r="B27" s="44" t="s">
-        <v>38</v>
-      </c>
-      <c r="C27" s="44" t="s">
-        <v>38</v>
-      </c>
-      <c r="D27" s="44" t="s">
-        <v>38</v>
-      </c>
-      <c r="E27" s="44" t="s">
-        <v>38</v>
-      </c>
-      <c r="F27" s="44" t="s">
-        <v>38</v>
+      <c r="B27" s="43" t="s">
+        <v>42</v>
+      </c>
+      <c r="C27" s="43" t="s">
+        <v>42</v>
+      </c>
+      <c r="D27" s="43" t="s">
+        <v>42</v>
+      </c>
+      <c r="E27" s="43" t="s">
+        <v>42</v>
+      </c>
+      <c r="F27" s="43" t="s">
+        <v>42</v>
       </c>
       <c r="G27" s="1"/>
       <c r="H27" s="23"/>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A28" s="22"/>
-      <c r="B28" s="43" t="s">
-        <v>43</v>
-      </c>
-      <c r="C28" s="43" t="s">
-        <v>43</v>
-      </c>
-      <c r="D28" s="43" t="s">
-        <v>43</v>
-      </c>
-      <c r="E28" s="43" t="s">
-        <v>43</v>
-      </c>
-      <c r="F28" s="43" t="s">
-        <v>43</v>
+      <c r="B28" s="44" t="s">
+        <v>38</v>
+      </c>
+      <c r="C28" s="44" t="s">
+        <v>38</v>
+      </c>
+      <c r="D28" s="44" t="s">
+        <v>38</v>
+      </c>
+      <c r="E28" s="44" t="s">
+        <v>38</v>
+      </c>
+      <c r="F28" s="44" t="s">
+        <v>38</v>
       </c>
       <c r="G28" s="1"/>
       <c r="H28" s="23"/>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A29" s="22"/>
-      <c r="B29" s="44" t="s">
-        <v>41</v>
-      </c>
-      <c r="C29" s="44" t="s">
-        <v>41</v>
-      </c>
-      <c r="D29" s="44" t="s">
-        <v>41</v>
-      </c>
-      <c r="E29" s="44" t="s">
-        <v>41</v>
-      </c>
-      <c r="F29" s="44" t="s">
-        <v>41</v>
+      <c r="B29" s="43" t="s">
+        <v>43</v>
+      </c>
+      <c r="C29" s="43" t="s">
+        <v>43</v>
+      </c>
+      <c r="D29" s="43" t="s">
+        <v>43</v>
+      </c>
+      <c r="E29" s="43" t="s">
+        <v>43</v>
+      </c>
+      <c r="F29" s="43" t="s">
+        <v>43</v>
       </c>
       <c r="G29" s="1"/>
       <c r="H29" s="23"/>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A30" s="22"/>
-      <c r="B30" s="43" t="s">
-        <v>44</v>
-      </c>
-      <c r="C30" s="43" t="s">
-        <v>44</v>
-      </c>
-      <c r="D30" s="43" t="s">
-        <v>44</v>
-      </c>
-      <c r="E30" s="43" t="s">
-        <v>44</v>
-      </c>
-      <c r="F30" s="43" t="s">
-        <v>44</v>
+      <c r="B30" s="44" t="s">
+        <v>41</v>
+      </c>
+      <c r="C30" s="44" t="s">
+        <v>41</v>
+      </c>
+      <c r="D30" s="44" t="s">
+        <v>41</v>
+      </c>
+      <c r="E30" s="44" t="s">
+        <v>41</v>
+      </c>
+      <c r="F30" s="44" t="s">
+        <v>41</v>
       </c>
       <c r="G30" s="1"/>
       <c r="H30" s="23"/>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A31" s="22"/>
-      <c r="B31" s="44" t="s">
-        <v>38</v>
-      </c>
-      <c r="C31" s="44" t="s">
-        <v>41</v>
-      </c>
-      <c r="D31" s="44" t="s">
-        <v>38</v>
-      </c>
-      <c r="E31" s="44" t="s">
-        <v>41</v>
-      </c>
-      <c r="F31" s="44" t="s">
-        <v>38</v>
+      <c r="B31" s="43" t="s">
+        <v>44</v>
+      </c>
+      <c r="C31" s="43" t="s">
+        <v>44</v>
+      </c>
+      <c r="D31" s="43" t="s">
+        <v>44</v>
+      </c>
+      <c r="E31" s="43" t="s">
+        <v>44</v>
+      </c>
+      <c r="F31" s="43" t="s">
+        <v>44</v>
       </c>
       <c r="G31" s="1"/>
       <c r="H31" s="23"/>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A32" s="22"/>
-      <c r="B32" s="43" t="s">
-        <v>45</v>
-      </c>
-      <c r="C32" s="43" t="s">
-        <v>46</v>
-      </c>
-      <c r="D32" s="43" t="s">
-        <v>45</v>
-      </c>
-      <c r="E32" s="43" t="s">
-        <v>46</v>
-      </c>
-      <c r="F32" s="43" t="s">
-        <v>45</v>
+      <c r="B32" s="44" t="s">
+        <v>38</v>
+      </c>
+      <c r="C32" s="44" t="s">
+        <v>41</v>
+      </c>
+      <c r="D32" s="44" t="s">
+        <v>38</v>
+      </c>
+      <c r="E32" s="44" t="s">
+        <v>41</v>
+      </c>
+      <c r="F32" s="44" t="s">
+        <v>38</v>
       </c>
       <c r="G32" s="1"/>
       <c r="H32" s="23"/>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A33" s="22"/>
-      <c r="B33" s="44" t="s">
-        <v>41</v>
-      </c>
-      <c r="C33" s="43"/>
-      <c r="D33" s="44" t="s">
-        <v>41</v>
-      </c>
-      <c r="E33" s="43"/>
-      <c r="F33" s="43"/>
+      <c r="B33" s="43" t="s">
+        <v>45</v>
+      </c>
+      <c r="C33" s="43" t="s">
+        <v>46</v>
+      </c>
+      <c r="D33" s="43" t="s">
+        <v>45</v>
+      </c>
+      <c r="E33" s="43" t="s">
+        <v>46</v>
+      </c>
+      <c r="F33" s="43" t="s">
+        <v>45</v>
+      </c>
       <c r="G33" s="1"/>
       <c r="H33" s="23"/>
     </row>
-    <row r="34" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="24"/>
-      <c r="B34" s="45" t="s">
+    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A34" s="22"/>
+      <c r="B34" s="44" t="s">
+        <v>41</v>
+      </c>
+      <c r="C34" s="43"/>
+      <c r="D34" s="44" t="s">
+        <v>41</v>
+      </c>
+      <c r="E34" s="43"/>
+      <c r="F34" s="43"/>
+      <c r="G34" s="1"/>
+      <c r="H34" s="23"/>
+    </row>
+    <row r="35" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A35" s="24"/>
+      <c r="B35" s="45" t="s">
         <v>46</v>
       </c>
-      <c r="C34" s="45"/>
-      <c r="D34" s="45" t="s">
+      <c r="C35" s="45"/>
+      <c r="D35" s="45" t="s">
         <v>46</v>
       </c>
-      <c r="E34" s="45"/>
-      <c r="F34" s="45"/>
-      <c r="G34" s="25"/>
-      <c r="H34" s="26"/>
-    </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A35" s="19" t="s">
+      <c r="E35" s="45"/>
+      <c r="F35" s="45"/>
+      <c r="G35" s="25"/>
+      <c r="H35" s="26"/>
+    </row>
+    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A36" s="19" t="s">
         <v>47</v>
       </c>
-      <c r="B35" s="20" t="s">
+      <c r="B36" s="20" t="s">
         <v>12</v>
       </c>
-      <c r="C35" s="20"/>
-      <c r="D35" s="20"/>
-      <c r="E35" s="20" t="s">
+      <c r="C36" s="20"/>
+      <c r="D36" s="20"/>
+      <c r="E36" s="20" t="s">
         <v>12</v>
       </c>
-      <c r="F35" s="20"/>
-      <c r="G35" s="20"/>
-      <c r="H35" s="21"/>
-    </row>
-    <row r="36" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A36" s="24"/>
-      <c r="B36" s="25" t="s">
+      <c r="F36" s="20"/>
+      <c r="G36" s="20"/>
+      <c r="H36" s="21"/>
+    </row>
+    <row r="37" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A37" s="24"/>
+      <c r="B37" s="25" t="s">
         <v>48</v>
       </c>
-      <c r="C36" s="25"/>
-      <c r="D36" s="25"/>
-      <c r="E36" s="25" t="s">
+      <c r="C37" s="25"/>
+      <c r="D37" s="25"/>
+      <c r="E37" s="25" t="s">
         <v>48</v>
       </c>
-      <c r="F36" s="25"/>
-      <c r="G36" s="25"/>
-      <c r="H36" s="26"/>
-    </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A37" s="19" t="s">
+      <c r="F37" s="25"/>
+      <c r="G37" s="25"/>
+      <c r="H37" s="26"/>
+    </row>
+    <row r="38" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A38" s="19" t="s">
         <v>49</v>
       </c>
-      <c r="B37" s="20"/>
-      <c r="C37" s="20" t="s">
+      <c r="B38" s="20"/>
+      <c r="C38" s="20" t="s">
         <v>12</v>
       </c>
-      <c r="D37" s="20"/>
-      <c r="E37" s="20"/>
-      <c r="F37" s="20"/>
-      <c r="G37" s="20" t="s">
+      <c r="D38" s="20"/>
+      <c r="E38" s="20"/>
+      <c r="F38" s="20"/>
+      <c r="G38" s="20" t="s">
         <v>12</v>
       </c>
-      <c r="H37" s="21" t="s">
+      <c r="H38" s="21" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="38" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A38" s="24"/>
-      <c r="B38" s="25"/>
-      <c r="C38" s="25" t="s">
+    <row r="39" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A39" s="24"/>
+      <c r="B39" s="25"/>
+      <c r="C39" s="25" t="s">
         <v>28</v>
       </c>
-      <c r="D38" s="25"/>
-      <c r="E38" s="25"/>
-      <c r="F38" s="25"/>
-      <c r="G38" s="25" t="s">
+      <c r="D39" s="25"/>
+      <c r="E39" s="25"/>
+      <c r="F39" s="25"/>
+      <c r="G39" s="25" t="s">
         <v>50</v>
       </c>
-      <c r="H38" s="26" t="s">
+      <c r="H39" s="26" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="39" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A39" s="38" t="s">
+    <row r="40" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A40" s="38" t="s">
         <v>52</v>
       </c>
-      <c r="B39" s="39"/>
-      <c r="C39" s="40"/>
-      <c r="D39" s="40"/>
-      <c r="E39" s="40"/>
-      <c r="F39" s="40"/>
-      <c r="G39" s="40"/>
-      <c r="H39" s="41"/>
-    </row>
-    <row r="40" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A40" s="15" t="s">
-        <v>53</v>
-      </c>
-      <c r="B40" s="27"/>
-      <c r="C40" s="28"/>
-      <c r="D40" s="28"/>
-      <c r="E40" s="28"/>
-      <c r="F40" s="28"/>
-      <c r="G40" s="28"/>
-      <c r="H40" s="29"/>
+      <c r="B40" s="39"/>
+      <c r="C40" s="40"/>
+      <c r="D40" s="40"/>
+      <c r="E40" s="40"/>
+      <c r="F40" s="40"/>
+      <c r="G40" s="40"/>
+      <c r="H40" s="41"/>
     </row>
     <row r="41" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A41" s="15" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B41" s="27"/>
       <c r="C41" s="28"/>
@@ -5196,297 +5260,297 @@
       <c r="G41" s="28"/>
       <c r="H41" s="29"/>
     </row>
-    <row r="42" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A42" s="19" t="s">
+    <row r="42" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A42" s="15" t="s">
+        <v>54</v>
+      </c>
+      <c r="B42" s="27"/>
+      <c r="C42" s="28"/>
+      <c r="D42" s="28"/>
+      <c r="E42" s="28"/>
+      <c r="F42" s="28"/>
+      <c r="G42" s="28"/>
+      <c r="H42" s="29"/>
+    </row>
+    <row r="43" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A43" s="19" t="s">
         <v>55</v>
       </c>
-      <c r="B42" s="20" t="s">
+      <c r="B43" s="20" t="s">
         <v>12</v>
       </c>
-      <c r="C42" s="20" t="s">
+      <c r="C43" s="20" t="s">
         <v>12</v>
       </c>
-      <c r="D42" s="20" t="s">
+      <c r="D43" s="20" t="s">
         <v>12</v>
       </c>
-      <c r="E42" s="20"/>
-      <c r="F42" s="20"/>
-      <c r="G42" s="20"/>
-      <c r="H42" s="21"/>
-    </row>
-    <row r="43" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A43" s="24"/>
-      <c r="B43" s="25" t="s">
+      <c r="E43" s="20"/>
+      <c r="F43" s="20"/>
+      <c r="G43" s="20"/>
+      <c r="H43" s="21"/>
+    </row>
+    <row r="44" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A44" s="24"/>
+      <c r="B44" s="25" t="s">
         <v>56</v>
       </c>
-      <c r="C43" s="25" t="s">
+      <c r="C44" s="25" t="s">
         <v>57</v>
       </c>
-      <c r="D43" s="25" t="s">
+      <c r="D44" s="25" t="s">
         <v>57</v>
       </c>
-      <c r="E43" s="25"/>
-      <c r="F43" s="25"/>
-      <c r="G43" s="25"/>
-      <c r="H43" s="26"/>
-    </row>
-    <row r="44" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A44" s="15" t="s">
+      <c r="E44" s="25"/>
+      <c r="F44" s="25"/>
+      <c r="G44" s="25"/>
+      <c r="H44" s="26"/>
+    </row>
+    <row r="45" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A45" s="15" t="s">
         <v>58</v>
       </c>
-      <c r="B44" s="27"/>
-      <c r="C44" s="28"/>
-      <c r="D44" s="28"/>
-      <c r="E44" s="28"/>
-      <c r="F44" s="28"/>
-      <c r="G44" s="28"/>
-      <c r="H44" s="29"/>
-    </row>
-    <row r="45" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A45" s="19" t="s">
+      <c r="B45" s="27"/>
+      <c r="C45" s="28"/>
+      <c r="D45" s="28"/>
+      <c r="E45" s="28"/>
+      <c r="F45" s="28"/>
+      <c r="G45" s="28"/>
+      <c r="H45" s="29"/>
+    </row>
+    <row r="46" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A46" s="19" t="s">
         <v>59</v>
       </c>
-      <c r="B45" s="42" t="s">
+      <c r="B46" s="42" t="s">
         <v>38</v>
       </c>
-      <c r="C45" s="42" t="s">
+      <c r="C46" s="42" t="s">
         <v>38</v>
       </c>
-      <c r="D45" s="42" t="s">
+      <c r="D46" s="42" t="s">
         <v>38</v>
       </c>
-      <c r="E45" s="42" t="s">
+      <c r="E46" s="42" t="s">
         <v>38</v>
       </c>
-      <c r="F45" s="42" t="s">
+      <c r="F46" s="42" t="s">
         <v>38</v>
       </c>
-      <c r="G45" s="20"/>
-      <c r="H45" s="21"/>
-    </row>
-    <row r="46" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A46" s="22"/>
-      <c r="B46" s="43" t="s">
-        <v>39</v>
-      </c>
-      <c r="C46" s="43" t="s">
-        <v>40</v>
-      </c>
-      <c r="D46" s="43" t="s">
-        <v>39</v>
-      </c>
-      <c r="E46" s="43" t="s">
-        <v>40</v>
-      </c>
-      <c r="F46" s="43" t="s">
-        <v>39</v>
-      </c>
-      <c r="G46" s="1"/>
-      <c r="H46" s="23"/>
+      <c r="G46" s="20"/>
+      <c r="H46" s="21"/>
     </row>
     <row r="47" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A47" s="22"/>
-      <c r="B47" s="44" t="s">
-        <v>41</v>
-      </c>
-      <c r="C47" s="44" t="s">
-        <v>41</v>
-      </c>
-      <c r="D47" s="44" t="s">
-        <v>41</v>
-      </c>
-      <c r="E47" s="44" t="s">
-        <v>41</v>
-      </c>
-      <c r="F47" s="44" t="s">
-        <v>41</v>
+      <c r="B47" s="43" t="s">
+        <v>39</v>
+      </c>
+      <c r="C47" s="43" t="s">
+        <v>40</v>
+      </c>
+      <c r="D47" s="43" t="s">
+        <v>39</v>
+      </c>
+      <c r="E47" s="43" t="s">
+        <v>40</v>
+      </c>
+      <c r="F47" s="43" t="s">
+        <v>39</v>
       </c>
       <c r="G47" s="1"/>
       <c r="H47" s="23"/>
     </row>
     <row r="48" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A48" s="22"/>
-      <c r="B48" s="43" t="s">
-        <v>42</v>
-      </c>
-      <c r="C48" s="43" t="s">
-        <v>42</v>
-      </c>
-      <c r="D48" s="43" t="s">
-        <v>42</v>
-      </c>
-      <c r="E48" s="43" t="s">
-        <v>42</v>
-      </c>
-      <c r="F48" s="43" t="s">
-        <v>42</v>
+      <c r="B48" s="44" t="s">
+        <v>41</v>
+      </c>
+      <c r="C48" s="44" t="s">
+        <v>41</v>
+      </c>
+      <c r="D48" s="44" t="s">
+        <v>41</v>
+      </c>
+      <c r="E48" s="44" t="s">
+        <v>41</v>
+      </c>
+      <c r="F48" s="44" t="s">
+        <v>41</v>
       </c>
       <c r="G48" s="1"/>
       <c r="H48" s="23"/>
     </row>
     <row r="49" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A49" s="22"/>
-      <c r="B49" s="44" t="s">
-        <v>38</v>
-      </c>
-      <c r="C49" s="44" t="s">
-        <v>38</v>
-      </c>
-      <c r="D49" s="44" t="s">
-        <v>38</v>
-      </c>
-      <c r="E49" s="44" t="s">
-        <v>38</v>
-      </c>
-      <c r="F49" s="44" t="s">
-        <v>38</v>
+      <c r="B49" s="43" t="s">
+        <v>42</v>
+      </c>
+      <c r="C49" s="43" t="s">
+        <v>42</v>
+      </c>
+      <c r="D49" s="43" t="s">
+        <v>42</v>
+      </c>
+      <c r="E49" s="43" t="s">
+        <v>42</v>
+      </c>
+      <c r="F49" s="43" t="s">
+        <v>42</v>
       </c>
       <c r="G49" s="1"/>
       <c r="H49" s="23"/>
     </row>
     <row r="50" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A50" s="22"/>
-      <c r="B50" s="43" t="s">
-        <v>60</v>
-      </c>
-      <c r="C50" s="43" t="s">
-        <v>60</v>
-      </c>
-      <c r="D50" s="43" t="s">
-        <v>60</v>
-      </c>
-      <c r="E50" s="43" t="s">
-        <v>60</v>
-      </c>
-      <c r="F50" s="43" t="s">
-        <v>60</v>
+      <c r="B50" s="44" t="s">
+        <v>38</v>
+      </c>
+      <c r="C50" s="44" t="s">
+        <v>38</v>
+      </c>
+      <c r="D50" s="44" t="s">
+        <v>38</v>
+      </c>
+      <c r="E50" s="44" t="s">
+        <v>38</v>
+      </c>
+      <c r="F50" s="44" t="s">
+        <v>38</v>
       </c>
       <c r="G50" s="1"/>
       <c r="H50" s="23"/>
     </row>
     <row r="51" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A51" s="22"/>
-      <c r="B51" s="44" t="s">
-        <v>41</v>
-      </c>
-      <c r="C51" s="44" t="s">
-        <v>41</v>
-      </c>
-      <c r="D51" s="44" t="s">
-        <v>41</v>
-      </c>
-      <c r="E51" s="44" t="s">
-        <v>41</v>
-      </c>
-      <c r="F51" s="44" t="s">
-        <v>41</v>
+      <c r="B51" s="43" t="s">
+        <v>60</v>
+      </c>
+      <c r="C51" s="43" t="s">
+        <v>60</v>
+      </c>
+      <c r="D51" s="43" t="s">
+        <v>60</v>
+      </c>
+      <c r="E51" s="43" t="s">
+        <v>60</v>
+      </c>
+      <c r="F51" s="43" t="s">
+        <v>60</v>
       </c>
       <c r="G51" s="1"/>
       <c r="H51" s="23"/>
     </row>
     <row r="52" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A52" s="22"/>
-      <c r="B52" s="43" t="s">
-        <v>44</v>
-      </c>
-      <c r="C52" s="43" t="s">
-        <v>44</v>
-      </c>
-      <c r="D52" s="43" t="s">
-        <v>44</v>
-      </c>
-      <c r="E52" s="43" t="s">
-        <v>44</v>
-      </c>
-      <c r="F52" s="43" t="s">
-        <v>44</v>
+      <c r="B52" s="44" t="s">
+        <v>41</v>
+      </c>
+      <c r="C52" s="44" t="s">
+        <v>41</v>
+      </c>
+      <c r="D52" s="44" t="s">
+        <v>41</v>
+      </c>
+      <c r="E52" s="44" t="s">
+        <v>41</v>
+      </c>
+      <c r="F52" s="44" t="s">
+        <v>41</v>
       </c>
       <c r="G52" s="1"/>
       <c r="H52" s="23"/>
     </row>
     <row r="53" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A53" s="22"/>
-      <c r="B53" s="44" t="s">
-        <v>41</v>
-      </c>
-      <c r="C53" s="44" t="s">
-        <v>38</v>
-      </c>
-      <c r="D53" s="44" t="s">
-        <v>41</v>
-      </c>
-      <c r="E53" s="44" t="s">
-        <v>38</v>
-      </c>
-      <c r="F53" s="44" t="s">
-        <v>38</v>
+      <c r="B53" s="43" t="s">
+        <v>44</v>
+      </c>
+      <c r="C53" s="43" t="s">
+        <v>44</v>
+      </c>
+      <c r="D53" s="43" t="s">
+        <v>44</v>
+      </c>
+      <c r="E53" s="43" t="s">
+        <v>44</v>
+      </c>
+      <c r="F53" s="43" t="s">
+        <v>44</v>
       </c>
       <c r="G53" s="1"/>
       <c r="H53" s="23"/>
     </row>
     <row r="54" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A54" s="22"/>
-      <c r="B54" s="43" t="s">
-        <v>46</v>
-      </c>
-      <c r="C54" s="43" t="s">
-        <v>45</v>
-      </c>
-      <c r="D54" s="43" t="s">
-        <v>46</v>
-      </c>
-      <c r="E54" s="43" t="s">
-        <v>45</v>
-      </c>
-      <c r="F54" s="43" t="s">
-        <v>45</v>
+      <c r="B54" s="44" t="s">
+        <v>41</v>
+      </c>
+      <c r="C54" s="44" t="s">
+        <v>38</v>
+      </c>
+      <c r="D54" s="44" t="s">
+        <v>41</v>
+      </c>
+      <c r="E54" s="44" t="s">
+        <v>38</v>
+      </c>
+      <c r="F54" s="44" t="s">
+        <v>38</v>
       </c>
       <c r="G54" s="1"/>
       <c r="H54" s="23"/>
     </row>
     <row r="55" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A55" s="22"/>
-      <c r="B55" s="43"/>
-      <c r="C55" s="44" t="s">
-        <v>41</v>
-      </c>
-      <c r="D55" s="43"/>
-      <c r="E55" s="44" t="s">
-        <v>41</v>
-      </c>
-      <c r="F55" s="43"/>
+      <c r="B55" s="43" t="s">
+        <v>46</v>
+      </c>
+      <c r="C55" s="43" t="s">
+        <v>45</v>
+      </c>
+      <c r="D55" s="43" t="s">
+        <v>46</v>
+      </c>
+      <c r="E55" s="43" t="s">
+        <v>45</v>
+      </c>
+      <c r="F55" s="43" t="s">
+        <v>45</v>
+      </c>
       <c r="G55" s="1"/>
       <c r="H55" s="23"/>
     </row>
-    <row r="56" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A56" s="24"/>
-      <c r="B56" s="45"/>
-      <c r="C56" s="45" t="s">
+    <row r="56" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A56" s="22"/>
+      <c r="B56" s="43"/>
+      <c r="C56" s="44" t="s">
+        <v>41</v>
+      </c>
+      <c r="D56" s="43"/>
+      <c r="E56" s="44" t="s">
+        <v>41</v>
+      </c>
+      <c r="F56" s="43"/>
+      <c r="G56" s="1"/>
+      <c r="H56" s="23"/>
+    </row>
+    <row r="57" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A57" s="24"/>
+      <c r="B57" s="45"/>
+      <c r="C57" s="45" t="s">
         <v>46</v>
       </c>
-      <c r="D56" s="45"/>
-      <c r="E56" s="45" t="s">
+      <c r="D57" s="45"/>
+      <c r="E57" s="45" t="s">
         <v>46</v>
       </c>
-      <c r="F56" s="45"/>
-      <c r="G56" s="25"/>
-      <c r="H56" s="26"/>
-    </row>
-    <row r="57" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A57" s="15" t="s">
-        <v>62</v>
-      </c>
-      <c r="B57" s="16"/>
-      <c r="C57" s="17"/>
-      <c r="D57" s="17"/>
-      <c r="E57" s="17"/>
-      <c r="F57" s="17"/>
-      <c r="G57" s="17"/>
-      <c r="H57" s="18"/>
+      <c r="F57" s="45"/>
+      <c r="G57" s="25"/>
+      <c r="H57" s="26"/>
     </row>
     <row r="58" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A58" s="15" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B58" s="16"/>
       <c r="C58" s="17"/>
@@ -5496,42 +5560,54 @@
       <c r="G58" s="17"/>
       <c r="H58" s="18"/>
     </row>
-    <row r="59" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="B59" s="14"/>
-      <c r="C59" s="14"/>
-      <c r="D59" s="14"/>
-      <c r="E59" s="14"/>
-      <c r="F59" s="14"/>
-      <c r="G59" s="14"/>
-      <c r="H59" s="14"/>
+    <row r="59" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A59" s="15" t="s">
+        <v>63</v>
+      </c>
+      <c r="B59" s="16"/>
+      <c r="C59" s="17"/>
+      <c r="D59" s="17"/>
+      <c r="E59" s="17"/>
+      <c r="F59" s="17"/>
+      <c r="G59" s="17"/>
+      <c r="H59" s="18"/>
+    </row>
+    <row r="60" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B60" s="14"/>
+      <c r="C60" s="14"/>
+      <c r="D60" s="14"/>
+      <c r="E60" s="14"/>
+      <c r="F60" s="14"/>
+      <c r="G60" s="14"/>
+      <c r="H60" s="14"/>
     </row>
   </sheetData>
   <mergeCells count="28">
     <mergeCell ref="B7:H7"/>
-    <mergeCell ref="B12:H12"/>
     <mergeCell ref="B13:H13"/>
+    <mergeCell ref="B14:H14"/>
+    <mergeCell ref="B16:H16"/>
     <mergeCell ref="B15:H15"/>
-    <mergeCell ref="B14:H14"/>
-    <mergeCell ref="B22:H22"/>
-    <mergeCell ref="B18:H18"/>
+    <mergeCell ref="B23:H23"/>
     <mergeCell ref="B19:H19"/>
-    <mergeCell ref="B9:H9"/>
+    <mergeCell ref="B20:H20"/>
     <mergeCell ref="B8:H8"/>
+    <mergeCell ref="B60:H60"/>
     <mergeCell ref="B59:H59"/>
     <mergeCell ref="B58:H58"/>
-    <mergeCell ref="B57:H57"/>
-    <mergeCell ref="B39:H39"/>
     <mergeCell ref="B40:H40"/>
     <mergeCell ref="B41:H41"/>
-    <mergeCell ref="B44:H44"/>
-    <mergeCell ref="A45:A56"/>
-    <mergeCell ref="A37:A38"/>
-    <mergeCell ref="A42:A43"/>
-    <mergeCell ref="A20:A21"/>
-    <mergeCell ref="A23:A34"/>
-    <mergeCell ref="A35:A36"/>
-    <mergeCell ref="A16:A17"/>
-    <mergeCell ref="A10:A11"/>
+    <mergeCell ref="B42:H42"/>
+    <mergeCell ref="B45:H45"/>
+    <mergeCell ref="A46:A57"/>
+    <mergeCell ref="A38:A39"/>
+    <mergeCell ref="A43:A44"/>
+    <mergeCell ref="A21:A22"/>
+    <mergeCell ref="A24:A35"/>
+    <mergeCell ref="A36:A37"/>
+    <mergeCell ref="A17:A18"/>
+    <mergeCell ref="A11:A12"/>
+    <mergeCell ref="A9:A10"/>
     <mergeCell ref="B2:H2"/>
     <mergeCell ref="B1:H1"/>
     <mergeCell ref="A5:A6"/>
@@ -6310,13 +6386,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D48D083B-579F-4396-8CFC-BBC1F0F4D773}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2DD39EA0-7005-4948-9532-0B8CEC916B0F}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F2630203-7D8D-43CE-86C7-C0680DAC53A9}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5DDC03C6-2F7D-4A10-96DA-69C85BFD333A}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F24F2F4E-E51C-4CDF-867F-CC2459314358}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E70FF7F0-400D-4287-9857-C20CEB30CADC}"/>
 </file>
</xml_diff>